<commit_message>
Add «ΠΑΝΤΑ MSRP» override; apply it to the three borderline items
OVERRIDES can now force a code to MSRP and ignore any customer SPA,
same effect as rule 2β, for items whose catalog category isn't
FR/RK/CA. Νίκος confirmed the three borderline lines from the 20/10
report belong in that group: SRB19BLY (rear cable manager, OU8),
GB4B1028TPI-1 (grounding bar, PC7), QAPP24BL (QuickNet blank panel,
FB8). All 54 report lines are now covered.

Checked that none of the existing override texts parse as the new
directive. Diff vs previous engine on the October inputs: exactly
these 3 lines move SPA -> MSRP, nothing else. test.js: 2924 rows,
890 changed, 23 ΓΙΑ_ΕΛΕΓΧΟ, tests and integrity pass; same in
Chromium. RULES V3.3 and team memo updated; demo rebuilt, no leaks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BzJGp7TZogkrcqXW4FbpaM
</commit_message>
<xml_diff>
--- a/html/params/ΠΑΡΑΜΕΤΡΟΙ_v6.xlsx
+++ b/html/params/ΠΑΡΑΜΕΤΡΟΙ_v6.xlsx
@@ -8960,11 +8960,11 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Υπερισχύουν των πάντων. «Τι επιβάλλουμε» καταλαβαίνει: «πακέτο = N», «μονάδα = N», «ΑΠΟΔΟΧΗ ΑΠΟΚΛΙΣΗΣ» (περνά τη Δ1). Μπορείς να γράψεις πολλά χωρισμένα με ;</v>
+        <v>Υπερισχύουν των πάντων. «Τι επιβάλλουμε» καταλαβαίνει: «πακέτο = N», «μονάδα = N», «ΑΠΟΔΟΧΗ ΑΠΟΚΛΙΣΗΣ» (περνά τη Δ1), «ΠΑΝΤΑ MSRP» (ποτέ SPA πελάτη, όπως ο κανόνας 2β). Μπορείς να γράψεις πολλά χωρισμένα με ;</v>
       </c>
     </row>
     <row r="2">
@@ -9103,9 +9103,60 @@
         <v>Report τιμολόγησης 20/10/2026</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>SRB19BLY</v>
+      </c>
+      <c r="B10" t="str">
+        <v>ΠΙΣΩ ΟΔΗΓΟΣ ΚΑΛ.19''</v>
+      </c>
+      <c r="C10" t="str">
+        <v>ΠΑΝΤΑ MSRP</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Παρελκόμενο rack: όχι SPA έργου πελάτη. Η κατηγορία καταλόγου (OU8/PC7/FB8) δεν είναι rack, γι'αυτό χρειάζεται εδώ.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Νίκος 27/10/2026</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>GB4B1028TPI-1</v>
+      </c>
+      <c r="B11" t="str">
+        <v>ΜΠΑΡΑ ΓΕΙΩΣΗΣ ΔΙΑΤΡ 6,4X102Χ610MM</v>
+      </c>
+      <c r="C11" t="str">
+        <v>ΠΑΝΤΑ MSRP</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Παρελκόμενο rack: όχι SPA έργου πελάτη. Η κατηγορία καταλόγου (OU8/PC7/FB8) δεν είναι rack, γι'αυτό χρειάζεται εδώ.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Νίκος 27/10/2026</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>QAPP24BL</v>
+      </c>
+      <c r="B12" t="str">
+        <v>P.PANEL KENO ΓΩΝΙΑΚΟ QUICKNET</v>
+      </c>
+      <c r="C12" t="str">
+        <v>ΠΑΝΤΑ MSRP</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Παρελκόμενο rack: όχι SPA έργου πελάτη. Η κατηγορία καταλόγου (OU8/PC7/FB8) δεν είναι rack, γι'αυτό χρειάζεται εδώ.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Νίκος 27/10/2026</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>